<commit_message>
docs: update candidate details and repository URL
</commit_message>
<xml_diff>
--- a/Assessment2_Submission_Workbook.xlsx
+++ b/Assessment2_Submission_Workbook.xlsx
@@ -515,7 +515,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>IncuBrix Candidate (PS2)</t>
+          <t>Ratchagan (PS2)</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Confirmed and Signed: IncuBrix Candidate</t>
+          <t>Confirmed and Signed: Ratchagan</t>
         </is>
       </c>
     </row>

</xml_diff>